<commit_message>
chore: actualización automática 2026-08-01
</commit_message>
<xml_diff>
--- a/Base_Andina_Ventas_Auto.xlsx
+++ b/Base_Andina_Ventas_Auto.xlsx
@@ -9037,7 +9037,7 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Kia</t>
+          <t>Kgm</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -9046,10 +9046,10 @@
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>1838</v>
+        <v>283</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>1838</v>
+        <v>283</v>
       </c>
     </row>
     <row r="13">
@@ -9066,19 +9066,19 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Maxus</t>
+          <t>Kia</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>China 🇨🇳</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>564</v>
+        <v>1838</v>
       </c>
       <c r="G13" t="n">
-        <v>564</v>
+        <v>1838</v>
       </c>
     </row>
     <row r="14">
@@ -9095,19 +9095,19 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Mazda</t>
+          <t>Maxus</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>778</v>
+        <v>564</v>
       </c>
       <c r="G14" s="2" t="n">
-        <v>778</v>
+        <v>564</v>
       </c>
     </row>
     <row r="15">
@@ -9124,19 +9124,19 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Mg</t>
+          <t>Mazda</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>China 🇨🇳</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>945</v>
+        <v>778</v>
       </c>
       <c r="G15" t="n">
-        <v>945</v>
+        <v>778</v>
       </c>
     </row>
     <row r="16">
@@ -9153,19 +9153,19 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Mitsubishi</t>
+          <t>Mg</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F16" s="2" t="n">
-        <v>1379</v>
+        <v>945</v>
       </c>
       <c r="G16" s="2" t="n">
-        <v>1379</v>
+        <v>945</v>
       </c>
     </row>
     <row r="17">
@@ -9182,7 +9182,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Nissan</t>
+          <t>Mitsubishi</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -9191,10 +9191,10 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>616</v>
+        <v>1379</v>
       </c>
       <c r="G17" t="n">
-        <v>616</v>
+        <v>1379</v>
       </c>
     </row>
     <row r="18">
@@ -9211,19 +9211,19 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Omoda</t>
+          <t>Nissan</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>China 🇨🇳</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F18" s="2" t="n">
-        <v>343</v>
+        <v>616</v>
       </c>
       <c r="G18" s="2" t="n">
-        <v>343</v>
+        <v>616</v>
       </c>
     </row>
     <row r="19">
@@ -9240,19 +9240,19 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Opel</t>
+          <t>Omoda</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>366</v>
+        <v>343</v>
       </c>
       <c r="G19" t="n">
-        <v>366</v>
+        <v>343</v>
       </c>
     </row>
     <row r="20">
@@ -9269,7 +9269,7 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Peugeot</t>
+          <t>Opel</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
@@ -9278,10 +9278,10 @@
         </is>
       </c>
       <c r="F20" s="2" t="n">
-        <v>1409</v>
+        <v>366</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>1409</v>
+        <v>366</v>
       </c>
     </row>
     <row r="21">
@@ -9298,7 +9298,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Ram</t>
+          <t>Peugeot</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -9307,10 +9307,10 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>356</v>
+        <v>1409</v>
       </c>
       <c r="G21" t="n">
-        <v>356</v>
+        <v>1409</v>
       </c>
     </row>
     <row r="22">
@@ -9327,7 +9327,7 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Ssangyong</t>
+          <t>Ram</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
@@ -9336,10 +9336,10 @@
         </is>
       </c>
       <c r="F22" s="2" t="n">
-        <v>283</v>
+        <v>356</v>
       </c>
       <c r="G22" s="2" t="n">
-        <v>283</v>
+        <v>356</v>
       </c>
     </row>
     <row r="23">
@@ -9760,7 +9760,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Kia</t>
+          <t>Kgm</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -9769,10 +9769,10 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>3180</v>
+        <v>534</v>
       </c>
       <c r="G37" t="n">
-        <v>1342</v>
+        <v>251</v>
       </c>
     </row>
     <row r="38">
@@ -9789,19 +9789,19 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Maxus</t>
+          <t>Kia</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>China 🇨🇳</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F38" s="2" t="n">
-        <v>1073</v>
+        <v>3180</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>509</v>
+        <v>1342</v>
       </c>
     </row>
     <row r="39">
@@ -9818,19 +9818,19 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Mazda</t>
+          <t>Maxus</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F39" t="n">
-        <v>1404</v>
+        <v>1073</v>
       </c>
       <c r="G39" t="n">
-        <v>626</v>
+        <v>509</v>
       </c>
     </row>
     <row r="40">
@@ -9847,19 +9847,19 @@
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Mg</t>
+          <t>Mazda</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>China 🇨🇳</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F40" s="2" t="n">
-        <v>1511</v>
+        <v>1404</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>566</v>
+        <v>626</v>
       </c>
     </row>
     <row r="41">
@@ -9876,19 +9876,19 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Mitsubishi</t>
+          <t>Mg</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F41" t="n">
-        <v>2275</v>
+        <v>1511</v>
       </c>
       <c r="G41" t="n">
-        <v>896</v>
+        <v>566</v>
       </c>
     </row>
     <row r="42">
@@ -9905,7 +9905,7 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Nissan</t>
+          <t>Mitsubishi</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
@@ -9914,10 +9914,10 @@
         </is>
       </c>
       <c r="F42" s="2" t="n">
-        <v>1105</v>
+        <v>2275</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>489</v>
+        <v>896</v>
       </c>
     </row>
     <row r="43">
@@ -9934,19 +9934,19 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Omoda</t>
+          <t>Nissan</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>China 🇨🇳</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F43" t="n">
-        <v>671</v>
+        <v>1105</v>
       </c>
       <c r="G43" t="n">
-        <v>328</v>
+        <v>489</v>
       </c>
     </row>
     <row r="44">
@@ -9963,19 +9963,19 @@
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Opel</t>
+          <t>Omoda</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F44" s="2" t="n">
-        <v>679</v>
+        <v>671</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>313</v>
+        <v>328</v>
       </c>
     </row>
     <row r="45">
@@ -9992,7 +9992,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Peugeot</t>
+          <t>Opel</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -10001,10 +10001,10 @@
         </is>
       </c>
       <c r="F45" t="n">
-        <v>2565</v>
+        <v>679</v>
       </c>
       <c r="G45" t="n">
-        <v>1156</v>
+        <v>313</v>
       </c>
     </row>
     <row r="46">
@@ -10021,7 +10021,7 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>Ram</t>
+          <t>Peugeot</t>
         </is>
       </c>
       <c r="E46" s="2" t="inlineStr">
@@ -10030,10 +10030,10 @@
         </is>
       </c>
       <c r="F46" s="2" t="n">
-        <v>595</v>
+        <v>2565</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>239</v>
+        <v>1156</v>
       </c>
     </row>
     <row r="47">
@@ -10050,7 +10050,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Ssangyong</t>
+          <t>Ram</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -10059,10 +10059,10 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>534</v>
+        <v>595</v>
       </c>
       <c r="G47" t="n">
-        <v>251</v>
+        <v>239</v>
       </c>
     </row>
     <row r="48">
@@ -10485,7 +10485,7 @@
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Kia</t>
+          <t>Kgm</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
@@ -10494,10 +10494,10 @@
         </is>
       </c>
       <c r="F62" s="2" t="n">
-        <v>4717</v>
+        <v>780</v>
       </c>
       <c r="G62" s="2" t="n">
-        <v>1537</v>
+        <v>246</v>
       </c>
     </row>
     <row r="63">
@@ -10514,19 +10514,19 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Maxus</t>
+          <t>Kia</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>China 🇨🇳</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F63" t="n">
-        <v>1528</v>
+        <v>4717</v>
       </c>
       <c r="G63" t="n">
-        <v>455</v>
+        <v>1537</v>
       </c>
     </row>
     <row r="64">
@@ -10543,19 +10543,19 @@
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Mazda</t>
+          <t>Maxus</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F64" s="2" t="n">
-        <v>2188</v>
+        <v>1528</v>
       </c>
       <c r="G64" s="2" t="n">
-        <v>784</v>
+        <v>455</v>
       </c>
     </row>
     <row r="65">
@@ -10572,19 +10572,19 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Mg</t>
+          <t>Mazda</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>China 🇨🇳</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F65" t="n">
-        <v>2147</v>
+        <v>2188</v>
       </c>
       <c r="G65" t="n">
-        <v>636</v>
+        <v>784</v>
       </c>
     </row>
     <row r="66">
@@ -10601,19 +10601,19 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Mitsubishi</t>
+          <t>Mg</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F66" s="2" t="n">
-        <v>3099</v>
+        <v>2147</v>
       </c>
       <c r="G66" s="2" t="n">
-        <v>824</v>
+        <v>636</v>
       </c>
     </row>
     <row r="67">
@@ -10630,7 +10630,7 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Nissan</t>
+          <t>Mitsubishi</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -10639,10 +10639,10 @@
         </is>
       </c>
       <c r="F67" t="n">
-        <v>1664</v>
+        <v>3099</v>
       </c>
       <c r="G67" t="n">
-        <v>559</v>
+        <v>824</v>
       </c>
     </row>
     <row r="68">
@@ -10659,19 +10659,19 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Omoda</t>
+          <t>Nissan</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>China 🇨🇳</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F68" s="2" t="n">
-        <v>1064</v>
+        <v>1664</v>
       </c>
       <c r="G68" s="2" t="n">
-        <v>393</v>
+        <v>559</v>
       </c>
     </row>
     <row r="69">
@@ -10688,19 +10688,19 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Opel</t>
+          <t>Omoda</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F69" t="n">
-        <v>1019</v>
+        <v>1064</v>
       </c>
       <c r="G69" t="n">
-        <v>340</v>
+        <v>393</v>
       </c>
     </row>
     <row r="70">
@@ -10717,7 +10717,7 @@
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Peugeot</t>
+          <t>Opel</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
@@ -10726,10 +10726,10 @@
         </is>
       </c>
       <c r="F70" s="2" t="n">
-        <v>3947</v>
+        <v>1019</v>
       </c>
       <c r="G70" s="2" t="n">
-        <v>1382</v>
+        <v>340</v>
       </c>
     </row>
     <row r="71">
@@ -10746,7 +10746,7 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Ram</t>
+          <t>Peugeot</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -10755,10 +10755,10 @@
         </is>
       </c>
       <c r="F71" t="n">
-        <v>993</v>
+        <v>3947</v>
       </c>
       <c r="G71" t="n">
-        <v>398</v>
+        <v>1382</v>
       </c>
     </row>
     <row r="72">
@@ -10775,7 +10775,7 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>Ssangyong</t>
+          <t>Ram</t>
         </is>
       </c>
       <c r="E72" s="2" t="inlineStr">
@@ -10784,10 +10784,10 @@
         </is>
       </c>
       <c r="F72" s="2" t="n">
-        <v>780</v>
+        <v>993</v>
       </c>
       <c r="G72" s="2" t="n">
-        <v>246</v>
+        <v>398</v>
       </c>
     </row>
     <row r="73">
@@ -11210,7 +11210,7 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Kia</t>
+          <t>Kgm</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
@@ -11219,10 +11219,10 @@
         </is>
       </c>
       <c r="F87" t="n">
-        <v>6327</v>
+        <v>1015</v>
       </c>
       <c r="G87" t="n">
-        <v>1610</v>
+        <v>235</v>
       </c>
     </row>
     <row r="88">
@@ -11239,19 +11239,19 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>Maxus</t>
+          <t>Kia</t>
         </is>
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>China 🇨🇳</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F88" s="2" t="n">
-        <v>2443</v>
+        <v>6327</v>
       </c>
       <c r="G88" s="2" t="n">
-        <v>915</v>
+        <v>1610</v>
       </c>
     </row>
     <row r="89">
@@ -11268,19 +11268,19 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Mazda</t>
+          <t>Maxus</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F89" t="n">
-        <v>2911</v>
+        <v>2443</v>
       </c>
       <c r="G89" t="n">
-        <v>723</v>
+        <v>915</v>
       </c>
     </row>
     <row r="90">
@@ -11297,19 +11297,19 @@
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>Mg</t>
+          <t>Mazda</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>China 🇨🇳</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F90" s="2" t="n">
-        <v>2788</v>
+        <v>2911</v>
       </c>
       <c r="G90" s="2" t="n">
-        <v>641</v>
+        <v>723</v>
       </c>
     </row>
     <row r="91">
@@ -11326,19 +11326,19 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Mitsubishi</t>
+          <t>Mg</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F91" t="n">
-        <v>4240</v>
+        <v>2788</v>
       </c>
       <c r="G91" t="n">
-        <v>1141</v>
+        <v>641</v>
       </c>
     </row>
     <row r="92">
@@ -11355,7 +11355,7 @@
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>Nissan</t>
+          <t>Mitsubishi</t>
         </is>
       </c>
       <c r="E92" s="2" t="inlineStr">
@@ -11364,10 +11364,10 @@
         </is>
       </c>
       <c r="F92" s="2" t="n">
-        <v>2213</v>
+        <v>4240</v>
       </c>
       <c r="G92" s="2" t="n">
-        <v>549</v>
+        <v>1141</v>
       </c>
     </row>
     <row r="93">
@@ -11384,19 +11384,19 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Omoda</t>
+          <t>Nissan</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>China 🇨🇳</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F93" t="n">
-        <v>1433</v>
+        <v>2213</v>
       </c>
       <c r="G93" t="n">
-        <v>369</v>
+        <v>549</v>
       </c>
     </row>
     <row r="94">
@@ -11413,19 +11413,19 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>Opel</t>
+          <t>Omoda</t>
         </is>
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F94" s="2" t="n">
-        <v>1379</v>
+        <v>1433</v>
       </c>
       <c r="G94" s="2" t="n">
-        <v>360</v>
+        <v>369</v>
       </c>
     </row>
     <row r="95">
@@ -11442,7 +11442,7 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Peugeot</t>
+          <t>Opel</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -11451,10 +11451,10 @@
         </is>
       </c>
       <c r="F95" t="n">
-        <v>5268</v>
+        <v>1379</v>
       </c>
       <c r="G95" t="n">
-        <v>1321</v>
+        <v>360</v>
       </c>
     </row>
     <row r="96">
@@ -11471,7 +11471,7 @@
       </c>
       <c r="D96" s="2" t="inlineStr">
         <is>
-          <t>Ram</t>
+          <t>Peugeot</t>
         </is>
       </c>
       <c r="E96" s="2" t="inlineStr">
@@ -11480,10 +11480,10 @@
         </is>
       </c>
       <c r="F96" s="2" t="n">
-        <v>1310</v>
+        <v>5268</v>
       </c>
       <c r="G96" s="2" t="n">
-        <v>317</v>
+        <v>1321</v>
       </c>
     </row>
     <row r="97">
@@ -11500,7 +11500,7 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Ssangyong</t>
+          <t>Ram</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
@@ -11509,10 +11509,10 @@
         </is>
       </c>
       <c r="F97" t="n">
-        <v>1015</v>
+        <v>1310</v>
       </c>
       <c r="G97" t="n">
-        <v>235</v>
+        <v>317</v>
       </c>
     </row>
     <row r="98">
@@ -11935,7 +11935,7 @@
       </c>
       <c r="D112" s="2" t="inlineStr">
         <is>
-          <t>Kia</t>
+          <t>Kgm</t>
         </is>
       </c>
       <c r="E112" s="2" t="inlineStr">
@@ -11944,10 +11944,10 @@
         </is>
       </c>
       <c r="F112" s="2" t="n">
-        <v>7735</v>
+        <v>1240</v>
       </c>
       <c r="G112" s="2" t="n">
-        <v>1408</v>
+        <v>225</v>
       </c>
     </row>
     <row r="113">
@@ -11964,19 +11964,19 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Maxus</t>
+          <t>Kia</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>China 🇨🇳</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F113" t="n">
-        <v>2967</v>
+        <v>7735</v>
       </c>
       <c r="G113" t="n">
-        <v>524</v>
+        <v>1408</v>
       </c>
     </row>
     <row r="114">
@@ -11993,19 +11993,19 @@
       </c>
       <c r="D114" s="2" t="inlineStr">
         <is>
-          <t>Mazda</t>
+          <t>Maxus</t>
         </is>
       </c>
       <c r="E114" s="2" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F114" s="2" t="n">
-        <v>3661</v>
+        <v>2967</v>
       </c>
       <c r="G114" s="2" t="n">
-        <v>750</v>
+        <v>524</v>
       </c>
     </row>
     <row r="115">
@@ -12022,19 +12022,19 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Mg</t>
+          <t>Mazda</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>China 🇨🇳</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F115" t="n">
-        <v>3428</v>
+        <v>3661</v>
       </c>
       <c r="G115" t="n">
-        <v>640</v>
+        <v>750</v>
       </c>
     </row>
     <row r="116">
@@ -12051,19 +12051,19 @@
       </c>
       <c r="D116" s="2" t="inlineStr">
         <is>
-          <t>Mitsubishi</t>
+          <t>Mg</t>
         </is>
       </c>
       <c r="E116" s="2" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F116" s="2" t="n">
-        <v>4993</v>
+        <v>3428</v>
       </c>
       <c r="G116" s="2" t="n">
-        <v>753</v>
+        <v>640</v>
       </c>
     </row>
     <row r="117">
@@ -12080,7 +12080,7 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Nissan</t>
+          <t>Mitsubishi</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -12089,10 +12089,10 @@
         </is>
       </c>
       <c r="F117" t="n">
-        <v>2767</v>
+        <v>4993</v>
       </c>
       <c r="G117" t="n">
-        <v>554</v>
+        <v>753</v>
       </c>
     </row>
     <row r="118">
@@ -12109,19 +12109,19 @@
       </c>
       <c r="D118" s="2" t="inlineStr">
         <is>
-          <t>Omoda</t>
+          <t>Nissan</t>
         </is>
       </c>
       <c r="E118" s="2" t="inlineStr">
         <is>
-          <t>China 🇨🇳</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F118" s="2" t="n">
-        <v>1888</v>
+        <v>2767</v>
       </c>
       <c r="G118" s="2" t="n">
-        <v>455</v>
+        <v>554</v>
       </c>
     </row>
     <row r="119">
@@ -12138,19 +12138,19 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Opel</t>
+          <t>Omoda</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F119" t="n">
-        <v>1693</v>
+        <v>1888</v>
       </c>
       <c r="G119" t="n">
-        <v>314</v>
+        <v>455</v>
       </c>
     </row>
     <row r="120">
@@ -12167,7 +12167,7 @@
       </c>
       <c r="D120" s="2" t="inlineStr">
         <is>
-          <t>Peugeot</t>
+          <t>Opel</t>
         </is>
       </c>
       <c r="E120" s="2" t="inlineStr">
@@ -12176,10 +12176,10 @@
         </is>
       </c>
       <c r="F120" s="2" t="n">
-        <v>6683</v>
+        <v>1693</v>
       </c>
       <c r="G120" s="2" t="n">
-        <v>1415</v>
+        <v>314</v>
       </c>
     </row>
     <row r="121">
@@ -12196,7 +12196,7 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Ram</t>
+          <t>Peugeot</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
@@ -12205,10 +12205,10 @@
         </is>
       </c>
       <c r="F121" t="n">
-        <v>1701</v>
+        <v>6683</v>
       </c>
       <c r="G121" t="n">
-        <v>391</v>
+        <v>1415</v>
       </c>
     </row>
     <row r="122">
@@ -12225,7 +12225,7 @@
       </c>
       <c r="D122" s="2" t="inlineStr">
         <is>
-          <t>Ssangyong</t>
+          <t>Ram</t>
         </is>
       </c>
       <c r="E122" s="2" t="inlineStr">
@@ -12234,10 +12234,10 @@
         </is>
       </c>
       <c r="F122" s="2" t="n">
-        <v>1240</v>
+        <v>1701</v>
       </c>
       <c r="G122" s="2" t="n">
-        <v>225</v>
+        <v>391</v>
       </c>
     </row>
     <row r="123">
@@ -12660,7 +12660,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Kia</t>
+          <t>Kgm</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
@@ -12669,10 +12669,10 @@
         </is>
       </c>
       <c r="F137" t="n">
-        <v>9042</v>
+        <v>1499</v>
       </c>
       <c r="G137" t="n">
-        <v>1307</v>
+        <v>259</v>
       </c>
     </row>
     <row r="138">
@@ -12689,19 +12689,19 @@
       </c>
       <c r="D138" s="2" t="inlineStr">
         <is>
-          <t>Maxus</t>
+          <t>Kia</t>
         </is>
       </c>
       <c r="E138" s="2" t="inlineStr">
         <is>
-          <t>China 🇨🇳</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F138" s="2" t="n">
-        <v>3425</v>
+        <v>9042</v>
       </c>
       <c r="G138" s="2" t="n">
-        <v>458</v>
+        <v>1307</v>
       </c>
     </row>
     <row r="139">
@@ -12718,19 +12718,19 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Mazda</t>
+          <t>Maxus</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F139" t="n">
-        <v>4458</v>
+        <v>3425</v>
       </c>
       <c r="G139" t="n">
-        <v>797</v>
+        <v>458</v>
       </c>
     </row>
     <row r="140">
@@ -12747,19 +12747,19 @@
       </c>
       <c r="D140" s="2" t="inlineStr">
         <is>
-          <t>Mg</t>
+          <t>Mazda</t>
         </is>
       </c>
       <c r="E140" s="2" t="inlineStr">
         <is>
-          <t>China 🇨🇳</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F140" s="2" t="n">
-        <v>4131</v>
+        <v>4458</v>
       </c>
       <c r="G140" s="2" t="n">
-        <v>703</v>
+        <v>797</v>
       </c>
     </row>
     <row r="141">
@@ -12776,19 +12776,19 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Mitsubishi</t>
+          <t>Mg</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F141" t="n">
-        <v>6097</v>
+        <v>4131</v>
       </c>
       <c r="G141" t="n">
-        <v>1104</v>
+        <v>703</v>
       </c>
     </row>
     <row r="142">
@@ -12805,7 +12805,7 @@
       </c>
       <c r="D142" s="2" t="inlineStr">
         <is>
-          <t>Nissan</t>
+          <t>Mitsubishi</t>
         </is>
       </c>
       <c r="E142" s="2" t="inlineStr">
@@ -12814,10 +12814,10 @@
         </is>
       </c>
       <c r="F142" s="2" t="n">
-        <v>3314</v>
+        <v>6097</v>
       </c>
       <c r="G142" s="2" t="n">
-        <v>547</v>
+        <v>1104</v>
       </c>
     </row>
     <row r="143">
@@ -12834,19 +12834,19 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Omoda</t>
+          <t>Nissan</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>China 🇨🇳</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F143" t="n">
-        <v>2334</v>
+        <v>3314</v>
       </c>
       <c r="G143" t="n">
-        <v>446</v>
+        <v>547</v>
       </c>
     </row>
     <row r="144">
@@ -12863,19 +12863,19 @@
       </c>
       <c r="D144" s="2" t="inlineStr">
         <is>
-          <t>Opel</t>
+          <t>Omoda</t>
         </is>
       </c>
       <c r="E144" s="2" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F144" s="2" t="n">
-        <v>1953</v>
+        <v>2334</v>
       </c>
       <c r="G144" s="2" t="n">
-        <v>260</v>
+        <v>446</v>
       </c>
     </row>
     <row r="145">
@@ -12892,7 +12892,7 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Peugeot</t>
+          <t>Opel</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
@@ -12901,10 +12901,10 @@
         </is>
       </c>
       <c r="F145" t="n">
-        <v>8141</v>
+        <v>1953</v>
       </c>
       <c r="G145" t="n">
-        <v>1458</v>
+        <v>260</v>
       </c>
     </row>
     <row r="146">
@@ -12921,7 +12921,7 @@
       </c>
       <c r="D146" s="2" t="inlineStr">
         <is>
-          <t>Ram</t>
+          <t>Peugeot</t>
         </is>
       </c>
       <c r="E146" s="2" t="inlineStr">
@@ -12930,10 +12930,10 @@
         </is>
       </c>
       <c r="F146" s="2" t="n">
-        <v>2039</v>
+        <v>8141</v>
       </c>
       <c r="G146" s="2" t="n">
-        <v>338</v>
+        <v>1458</v>
       </c>
     </row>
     <row r="147">
@@ -12950,7 +12950,7 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Ssangyong</t>
+          <t>Ram</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
@@ -12959,10 +12959,10 @@
         </is>
       </c>
       <c r="F147" t="n">
-        <v>1499</v>
+        <v>2039</v>
       </c>
       <c r="G147" t="n">
-        <v>259</v>
+        <v>338</v>
       </c>
     </row>
     <row r="148">
@@ -13385,7 +13385,7 @@
       </c>
       <c r="D162" s="2" t="inlineStr">
         <is>
-          <t>Kia</t>
+          <t>Kgm</t>
         </is>
       </c>
       <c r="E162" s="2" t="inlineStr">
@@ -13394,10 +13394,10 @@
         </is>
       </c>
       <c r="F162" s="2" t="n">
-        <v>10678</v>
+        <v>1789</v>
       </c>
       <c r="G162" s="2" t="n">
-        <v>1636</v>
+        <v>290</v>
       </c>
     </row>
     <row r="163">
@@ -13414,19 +13414,19 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>Maxus</t>
+          <t>Kia</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>China 🇨🇳</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F163" t="n">
-        <v>3947</v>
+        <v>10678</v>
       </c>
       <c r="G163" t="n">
-        <v>522</v>
+        <v>1636</v>
       </c>
     </row>
     <row r="164">
@@ -13443,19 +13443,19 @@
       </c>
       <c r="D164" s="2" t="inlineStr">
         <is>
-          <t>Mazda</t>
+          <t>Maxus</t>
         </is>
       </c>
       <c r="E164" s="2" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F164" s="2" t="n">
-        <v>5316</v>
+        <v>3947</v>
       </c>
       <c r="G164" s="2" t="n">
-        <v>858</v>
+        <v>522</v>
       </c>
     </row>
     <row r="165">
@@ -13472,19 +13472,19 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>Mg</t>
+          <t>Mazda</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>China 🇨🇳</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F165" t="n">
-        <v>4832</v>
+        <v>5316</v>
       </c>
       <c r="G165" t="n">
-        <v>701</v>
+        <v>858</v>
       </c>
     </row>
     <row r="166">
@@ -13501,19 +13501,19 @@
       </c>
       <c r="D166" s="2" t="inlineStr">
         <is>
-          <t>Mitsubishi</t>
+          <t>Mg</t>
         </is>
       </c>
       <c r="E166" s="2" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F166" s="2" t="n">
-        <v>7023</v>
+        <v>4832</v>
       </c>
       <c r="G166" s="2" t="n">
-        <v>926</v>
+        <v>701</v>
       </c>
     </row>
     <row r="167">
@@ -13530,7 +13530,7 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>Nissan</t>
+          <t>Mitsubishi</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
@@ -13539,10 +13539,10 @@
         </is>
       </c>
       <c r="F167" t="n">
-        <v>3998</v>
+        <v>7023</v>
       </c>
       <c r="G167" t="n">
-        <v>684</v>
+        <v>926</v>
       </c>
     </row>
     <row r="168">
@@ -13559,19 +13559,19 @@
       </c>
       <c r="D168" s="2" t="inlineStr">
         <is>
-          <t>Omoda</t>
+          <t>Nissan</t>
         </is>
       </c>
       <c r="E168" s="2" t="inlineStr">
         <is>
-          <t>China 🇨🇳</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F168" s="2" t="n">
-        <v>2771</v>
+        <v>3998</v>
       </c>
       <c r="G168" s="2" t="n">
-        <v>437</v>
+        <v>684</v>
       </c>
     </row>
     <row r="169">
@@ -13588,19 +13588,19 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>Opel</t>
+          <t>Omoda</t>
         </is>
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F169" t="n">
-        <v>2108</v>
+        <v>2771</v>
       </c>
       <c r="G169" t="n">
-        <v>155</v>
+        <v>437</v>
       </c>
     </row>
     <row r="170">
@@ -13617,7 +13617,7 @@
       </c>
       <c r="D170" s="2" t="inlineStr">
         <is>
-          <t>Peugeot</t>
+          <t>Opel</t>
         </is>
       </c>
       <c r="E170" s="2" t="inlineStr">
@@ -13626,10 +13626,10 @@
         </is>
       </c>
       <c r="F170" s="2" t="n">
-        <v>9401</v>
+        <v>2108</v>
       </c>
       <c r="G170" s="2" t="n">
-        <v>1260</v>
+        <v>155</v>
       </c>
     </row>
     <row r="171">
@@ -13646,7 +13646,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>Ram</t>
+          <t>Peugeot</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
@@ -13655,10 +13655,10 @@
         </is>
       </c>
       <c r="F171" t="n">
-        <v>2392</v>
+        <v>9401</v>
       </c>
       <c r="G171" t="n">
-        <v>353</v>
+        <v>1260</v>
       </c>
     </row>
     <row r="172">
@@ -13675,7 +13675,7 @@
       </c>
       <c r="D172" s="2" t="inlineStr">
         <is>
-          <t>Ssangyong</t>
+          <t>Ram</t>
         </is>
       </c>
       <c r="E172" s="2" t="inlineStr">
@@ -13684,10 +13684,10 @@
         </is>
       </c>
       <c r="F172" s="2" t="n">
-        <v>1789</v>
+        <v>2392</v>
       </c>
       <c r="G172" s="2" t="n">
-        <v>290</v>
+        <v>353</v>
       </c>
     </row>
     <row r="173">
@@ -16782,7 +16782,7 @@
       </c>
       <c r="D281" t="inlineStr">
         <is>
-          <t>Dfm</t>
+          <t>Dfsk</t>
         </is>
       </c>
       <c r="E281" t="inlineStr">
@@ -21001,7 +21001,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G584"/>
+  <dimension ref="A1:G604"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -27419,12 +27419,12 @@
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>Gwm</t>
+          <t>Great Wall</t>
         </is>
       </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F227" t="n">
@@ -27986,12 +27986,12 @@
       </c>
       <c r="D248" s="2" t="inlineStr">
         <is>
-          <t>Gwm</t>
+          <t>Great Wall</t>
         </is>
       </c>
       <c r="E248" s="2" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F248" s="2" t="n">
@@ -28538,12 +28538,12 @@
       </c>
       <c r="D268" s="2" t="inlineStr">
         <is>
-          <t>Gwm</t>
+          <t>Great Wall</t>
         </is>
       </c>
       <c r="E268" s="2" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F268" s="2" t="n">
@@ -29145,12 +29145,12 @@
       </c>
       <c r="D289" t="inlineStr">
         <is>
-          <t>Gwm</t>
+          <t>Great Wall</t>
         </is>
       </c>
       <c r="E289" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F289" t="n">
@@ -29696,12 +29696,12 @@
       </c>
       <c r="D308" s="2" t="inlineStr">
         <is>
-          <t>Gwm</t>
+          <t>Great Wall</t>
         </is>
       </c>
       <c r="E308" s="2" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F308" s="2" t="n">
@@ -30262,12 +30262,12 @@
       </c>
       <c r="D328" s="2" t="inlineStr">
         <is>
-          <t>Gwm</t>
+          <t>Great Wall</t>
         </is>
       </c>
       <c r="E328" s="2" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F328" s="2" t="n">
@@ -30814,12 +30814,12 @@
       </c>
       <c r="D348" s="2" t="inlineStr">
         <is>
-          <t>Gwm</t>
+          <t>Great Wall</t>
         </is>
       </c>
       <c r="E348" s="2" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F348" s="2" t="n">
@@ -31392,12 +31392,12 @@
       </c>
       <c r="D368" s="2" t="inlineStr">
         <is>
-          <t>Gwm</t>
+          <t>Great Wall</t>
         </is>
       </c>
       <c r="E368" s="2" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F368" s="2" t="n">
@@ -31972,12 +31972,12 @@
       </c>
       <c r="D388" s="2" t="inlineStr">
         <is>
-          <t>Gwm</t>
+          <t>Great Wall</t>
         </is>
       </c>
       <c r="E388" s="2" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F388" s="2" t="n">
@@ -32552,12 +32552,12 @@
       </c>
       <c r="D408" s="2" t="inlineStr">
         <is>
-          <t>Gwm</t>
+          <t>Great Wall</t>
         </is>
       </c>
       <c r="E408" s="2" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F408" s="2" t="n">
@@ -33132,12 +33132,12 @@
       </c>
       <c r="D428" s="2" t="inlineStr">
         <is>
-          <t>Gwm</t>
+          <t>Great Wall</t>
         </is>
       </c>
       <c r="E428" s="2" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F428" s="2" t="n">
@@ -33712,12 +33712,12 @@
       </c>
       <c r="D448" s="2" t="inlineStr">
         <is>
-          <t>Gwm</t>
+          <t>Great Wall</t>
         </is>
       </c>
       <c r="E448" s="2" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F448" s="2" t="n">
@@ -34319,12 +34319,12 @@
       </c>
       <c r="D469" t="inlineStr">
         <is>
-          <t>Gwm</t>
+          <t>Great Wall</t>
         </is>
       </c>
       <c r="E469" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F469" t="n">
@@ -35011,12 +35011,12 @@
       </c>
       <c r="D493" t="inlineStr">
         <is>
-          <t>Gwm</t>
+          <t>Great Wall</t>
         </is>
       </c>
       <c r="E493" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F493" t="n">
@@ -35591,12 +35591,12 @@
       </c>
       <c r="D513" t="inlineStr">
         <is>
-          <t>Gwm</t>
+          <t>Great Wall</t>
         </is>
       </c>
       <c r="E513" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F513" t="n">
@@ -36171,12 +36171,12 @@
       </c>
       <c r="D533" t="inlineStr">
         <is>
-          <t>Gwm</t>
+          <t>Great Wall</t>
         </is>
       </c>
       <c r="E533" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F533" t="n">
@@ -36751,12 +36751,12 @@
       </c>
       <c r="D553" t="inlineStr">
         <is>
-          <t>Gwm</t>
+          <t>Great Wall</t>
         </is>
       </c>
       <c r="E553" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F553" t="n">
@@ -37329,12 +37329,12 @@
       </c>
       <c r="D573" t="inlineStr">
         <is>
-          <t>Gwm</t>
+          <t>Great Wall</t>
         </is>
       </c>
       <c r="E573" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F573" t="n">
@@ -37659,6 +37659,584 @@
       </c>
       <c r="G584" s="2" t="n">
         <v>224</v>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B585" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C585" t="n">
+        <v>6</v>
+      </c>
+      <c r="D585" t="inlineStr">
+        <is>
+          <t>Byd</t>
+        </is>
+      </c>
+      <c r="E585" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F585" t="n">
+        <v>2490</v>
+      </c>
+      <c r="G585" t="n">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B586" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C586" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D586" s="2" t="inlineStr">
+        <is>
+          <t>Changan</t>
+        </is>
+      </c>
+      <c r="E586" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F586" s="2" t="n">
+        <v>1451</v>
+      </c>
+      <c r="G586" s="2" t="n">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B587" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C587" t="n">
+        <v>6</v>
+      </c>
+      <c r="D587" t="inlineStr">
+        <is>
+          <t>Chery</t>
+        </is>
+      </c>
+      <c r="E587" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F587" t="n">
+        <v>3785</v>
+      </c>
+      <c r="G587" t="n">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B588" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C588" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D588" s="2" t="inlineStr">
+        <is>
+          <t>Chevrolet</t>
+        </is>
+      </c>
+      <c r="E588" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F588" s="2" t="n">
+        <v>9341</v>
+      </c>
+      <c r="G588" s="2" t="n">
+        <v>1609</v>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B589" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C589" t="n">
+        <v>6</v>
+      </c>
+      <c r="D589" t="inlineStr">
+        <is>
+          <t>Dfsk</t>
+        </is>
+      </c>
+      <c r="E589" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F589" t="n">
+        <v>2228</v>
+      </c>
+      <c r="G589" t="n">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B590" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C590" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D590" s="2" t="inlineStr">
+        <is>
+          <t>Dongfeng</t>
+        </is>
+      </c>
+      <c r="E590" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F590" s="2" t="n">
+        <v>2780</v>
+      </c>
+      <c r="G590" s="2" t="n">
+        <v>533</v>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B591" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C591" t="n">
+        <v>6</v>
+      </c>
+      <c r="D591" t="inlineStr">
+        <is>
+          <t>Foton</t>
+        </is>
+      </c>
+      <c r="E591" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F591" t="n">
+        <v>1341</v>
+      </c>
+      <c r="G591" t="n">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B592" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C592" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D592" s="2" t="inlineStr">
+        <is>
+          <t>Great Wall</t>
+        </is>
+      </c>
+      <c r="E592" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F592" s="2" t="n">
+        <v>4329</v>
+      </c>
+      <c r="G592" s="2" t="n">
+        <v>821</v>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B593" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C593" t="n">
+        <v>6</v>
+      </c>
+      <c r="D593" t="inlineStr">
+        <is>
+          <t>Hino</t>
+        </is>
+      </c>
+      <c r="E593" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F593" t="n">
+        <v>1033</v>
+      </c>
+      <c r="G593" t="n">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B594" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C594" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D594" s="2" t="inlineStr">
+        <is>
+          <t>Hyundai</t>
+        </is>
+      </c>
+      <c r="E594" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F594" s="2" t="n">
+        <v>4232</v>
+      </c>
+      <c r="G594" s="2" t="n">
+        <v>630</v>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B595" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C595" t="n">
+        <v>6</v>
+      </c>
+      <c r="D595" t="inlineStr">
+        <is>
+          <t>Jac</t>
+        </is>
+      </c>
+      <c r="E595" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F595" t="n">
+        <v>2773</v>
+      </c>
+      <c r="G595" t="n">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B596" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C596" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D596" s="2" t="inlineStr">
+        <is>
+          <t>Jetour</t>
+        </is>
+      </c>
+      <c r="E596" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F596" s="2" t="n">
+        <v>1817</v>
+      </c>
+      <c r="G596" s="2" t="n">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B597" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C597" t="n">
+        <v>6</v>
+      </c>
+      <c r="D597" t="inlineStr">
+        <is>
+          <t>Kia</t>
+        </is>
+      </c>
+      <c r="E597" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F597" t="n">
+        <v>12512</v>
+      </c>
+      <c r="G597" t="n">
+        <v>2271</v>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B598" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C598" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D598" s="2" t="inlineStr">
+        <is>
+          <t>Mazda</t>
+        </is>
+      </c>
+      <c r="E598" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F598" s="2" t="n">
+        <v>1733</v>
+      </c>
+      <c r="G598" s="2" t="n">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B599" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C599" t="n">
+        <v>6</v>
+      </c>
+      <c r="D599" t="inlineStr">
+        <is>
+          <t>Mg</t>
+        </is>
+      </c>
+      <c r="E599" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F599" t="n">
+        <v>1007</v>
+      </c>
+      <c r="G599" t="inlineStr"/>
+    </row>
+    <row r="600">
+      <c r="A600" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B600" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C600" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D600" s="2" t="inlineStr">
+        <is>
+          <t>Renault</t>
+        </is>
+      </c>
+      <c r="E600" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F600" s="2" t="n">
+        <v>1089</v>
+      </c>
+      <c r="G600" s="2" t="n">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B601" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C601" t="n">
+        <v>6</v>
+      </c>
+      <c r="D601" t="inlineStr">
+        <is>
+          <t>Sinotruk</t>
+        </is>
+      </c>
+      <c r="E601" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F601" t="n">
+        <v>2571</v>
+      </c>
+      <c r="G601" t="n">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B602" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C602" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D602" s="2" t="inlineStr">
+        <is>
+          <t>Suzuki</t>
+        </is>
+      </c>
+      <c r="E602" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F602" s="2" t="n">
+        <v>2311</v>
+      </c>
+      <c r="G602" s="2" t="n">
+        <v>436</v>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B603" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C603" t="n">
+        <v>6</v>
+      </c>
+      <c r="D603" t="inlineStr">
+        <is>
+          <t>Toyota</t>
+        </is>
+      </c>
+      <c r="E603" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F603" t="n">
+        <v>3808</v>
+      </c>
+      <c r="G603" t="n">
+        <v>764</v>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B604" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C604" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D604" s="2" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="E604" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F604" s="2" t="n">
+        <v>1616</v>
+      </c>
+      <c r="G604" s="2" t="n">
+        <v>294</v>
       </c>
     </row>
   </sheetData>
@@ -47360,7 +47938,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G60"/>
+  <dimension ref="A1:G70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -48805,14 +49383,14 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Rep. Dominicana</t>
+          <t>Guatemala</t>
         </is>
       </c>
       <c r="B51" t="n">
         <v>2026</v>
       </c>
       <c r="C51" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
@@ -48825,52 +49403,56 @@
         </is>
       </c>
       <c r="F51" t="n">
-        <v>1155</v>
-      </c>
-      <c r="G51" t="inlineStr"/>
+        <v>1842</v>
+      </c>
+      <c r="G51" t="n">
+        <v>328</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>Rep. Dominicana</t>
+          <t>Guatemala</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
         <v>2026</v>
       </c>
       <c r="C52" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>Chevrolet</t>
+          <t>Foton</t>
         </is>
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F52" s="2" t="n">
-        <v>728</v>
-      </c>
-      <c r="G52" s="2" t="inlineStr"/>
+        <v>1447</v>
+      </c>
+      <c r="G52" s="2" t="n">
+        <v>218</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Rep. Dominicana</t>
+          <t>Guatemala</t>
         </is>
       </c>
       <c r="B53" t="n">
         <v>2026</v>
       </c>
       <c r="C53" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Honda</t>
+          <t>Hino</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
@@ -48879,25 +49461,27 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>475</v>
-      </c>
-      <c r="G53" t="inlineStr"/>
+        <v>1501</v>
+      </c>
+      <c r="G53" t="n">
+        <v>251</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>Rep. Dominicana</t>
+          <t>Guatemala</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
         <v>2026</v>
       </c>
       <c r="C54" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>Hyundai</t>
+          <t>Isuzu</t>
         </is>
       </c>
       <c r="E54" s="2" t="inlineStr">
@@ -48906,79 +49490,85 @@
         </is>
       </c>
       <c r="F54" s="2" t="n">
-        <v>1618</v>
-      </c>
-      <c r="G54" s="2" t="inlineStr"/>
+        <v>3673</v>
+      </c>
+      <c r="G54" s="2" t="n">
+        <v>628</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Rep. Dominicana</t>
+          <t>Guatemala</t>
         </is>
       </c>
       <c r="B55" t="n">
         <v>2026</v>
       </c>
       <c r="C55" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Isuzu</t>
+          <t>Jac</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F55" t="n">
-        <v>1292</v>
-      </c>
-      <c r="G55" t="inlineStr"/>
+        <v>2204</v>
+      </c>
+      <c r="G55" t="n">
+        <v>354</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>Rep. Dominicana</t>
+          <t>Guatemala</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
         <v>2026</v>
       </c>
       <c r="C56" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>Jetour</t>
+          <t>Kia</t>
         </is>
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>China 🇨🇳</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F56" s="2" t="n">
-        <v>469</v>
-      </c>
-      <c r="G56" s="2" t="inlineStr"/>
+        <v>1863</v>
+      </c>
+      <c r="G56" s="2" t="n">
+        <v>295</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Rep. Dominicana</t>
+          <t>Guatemala</t>
         </is>
       </c>
       <c r="B57" t="n">
         <v>2026</v>
       </c>
       <c r="C57" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Kia</t>
+          <t>Mitsubishi</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -48987,25 +49577,27 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>1566</v>
-      </c>
-      <c r="G57" t="inlineStr"/>
+        <v>2283</v>
+      </c>
+      <c r="G57" t="n">
+        <v>392</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>Rep. Dominicana</t>
+          <t>Guatemala</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
         <v>2026</v>
       </c>
       <c r="C58" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>Nissan</t>
+          <t>Suzuki</t>
         </is>
       </c>
       <c r="E58" s="2" t="inlineStr">
@@ -49014,25 +49606,27 @@
         </is>
       </c>
       <c r="F58" s="2" t="n">
-        <v>657</v>
-      </c>
-      <c r="G58" s="2" t="inlineStr"/>
+        <v>1979</v>
+      </c>
+      <c r="G58" s="2" t="n">
+        <v>332</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Rep. Dominicana</t>
+          <t>Guatemala</t>
         </is>
       </c>
       <c r="B59" t="n">
         <v>2026</v>
       </c>
       <c r="C59" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Suzuki</t>
+          <t>Toyota</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -49041,36 +49635,310 @@
         </is>
       </c>
       <c r="F59" t="n">
-        <v>831</v>
-      </c>
-      <c r="G59" t="inlineStr"/>
+        <v>9163</v>
+      </c>
+      <c r="G59" t="n">
+        <v>1633</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>Rep. Dominicana</t>
+          <t>Guatemala</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
         <v>2026</v>
       </c>
       <c r="C60" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="n">
+        <v>1020</v>
+      </c>
+      <c r="G60" s="2" t="n">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Rep. Dominicana</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C61" t="n">
         <v>5</v>
       </c>
-      <c r="D60" s="2" t="inlineStr">
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Changan</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F61" t="n">
+        <v>1155</v>
+      </c>
+      <c r="G61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Rep. Dominicana</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C62" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Chevrolet</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="n">
+        <v>728</v>
+      </c>
+      <c r="G62" s="2" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Rep. Dominicana</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C63" t="n">
+        <v>5</v>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Honda</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F63" t="n">
+        <v>475</v>
+      </c>
+      <c r="G63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Rep. Dominicana</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C64" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Hyundai</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="n">
+        <v>1618</v>
+      </c>
+      <c r="G64" s="2" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Rep. Dominicana</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C65" t="n">
+        <v>5</v>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Isuzu</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F65" t="n">
+        <v>1292</v>
+      </c>
+      <c r="G65" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Rep. Dominicana</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C66" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Jetour</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="n">
+        <v>469</v>
+      </c>
+      <c r="G66" s="2" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Rep. Dominicana</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C67" t="n">
+        <v>5</v>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>Kia</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F67" t="n">
+        <v>1566</v>
+      </c>
+      <c r="G67" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>Rep. Dominicana</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C68" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>Nissan</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="n">
+        <v>657</v>
+      </c>
+      <c r="G68" s="2" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Rep. Dominicana</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C69" t="n">
+        <v>5</v>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>Suzuki</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>831</v>
+      </c>
+      <c r="G69" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>Rep. Dominicana</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C70" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
         <is>
           <t>Toyota</t>
         </is>
       </c>
-      <c r="E60" s="2" t="inlineStr">
-        <is>
-          <t>Otra</t>
-        </is>
-      </c>
-      <c r="F60" s="2" t="n">
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="n">
         <v>2304</v>
       </c>
-      <c r="G60" s="2" t="inlineStr"/>
+      <c r="G70" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: actualización automática 2026-08-15
</commit_message>
<xml_diff>
--- a/Base_Andina_Ventas_Auto.xlsx
+++ b/Base_Andina_Ventas_Auto.xlsx
@@ -3414,7 +3414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G181"/>
+  <dimension ref="A1:G191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -8673,6 +8673,296 @@
         <v>1798</v>
       </c>
     </row>
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="B182" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C182" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D182" s="2" t="inlineStr">
+        <is>
+          <t>Changan</t>
+        </is>
+      </c>
+      <c r="E182" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F182" s="2" t="n">
+        <v>4932</v>
+      </c>
+      <c r="G182" s="2" t="n">
+        <v>571</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="B183" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C183" t="n">
+        <v>7</v>
+      </c>
+      <c r="D183" t="inlineStr">
+        <is>
+          <t>Chery</t>
+        </is>
+      </c>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F183" t="n">
+        <v>3772</v>
+      </c>
+      <c r="G183" t="n">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="B184" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C184" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D184" s="2" t="inlineStr">
+        <is>
+          <t>Ford</t>
+        </is>
+      </c>
+      <c r="E184" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F184" s="2" t="n">
+        <v>3654</v>
+      </c>
+      <c r="G184" s="2" t="n">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="B185" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C185" t="n">
+        <v>7</v>
+      </c>
+      <c r="D185" t="inlineStr">
+        <is>
+          <t>Geely</t>
+        </is>
+      </c>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F185" t="n">
+        <v>6057</v>
+      </c>
+      <c r="G185" t="n">
+        <v>927</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="B186" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C186" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D186" s="2" t="inlineStr">
+        <is>
+          <t>Hyundai</t>
+        </is>
+      </c>
+      <c r="E186" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F186" s="2" t="n">
+        <v>6570</v>
+      </c>
+      <c r="G186" s="2" t="n">
+        <v>817</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="B187" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C187" t="n">
+        <v>7</v>
+      </c>
+      <c r="D187" t="inlineStr">
+        <is>
+          <t>Jac</t>
+        </is>
+      </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F187" t="n">
+        <v>2690</v>
+      </c>
+      <c r="G187" t="n">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="B188" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C188" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D188" s="2" t="inlineStr">
+        <is>
+          <t>Jetour</t>
+        </is>
+      </c>
+      <c r="E188" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F188" s="2" t="n">
+        <v>8641</v>
+      </c>
+      <c r="G188" s="2" t="n">
+        <v>1217</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="B189" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C189" t="n">
+        <v>7</v>
+      </c>
+      <c r="D189" t="inlineStr">
+        <is>
+          <t>Kia</t>
+        </is>
+      </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F189" t="n">
+        <v>6617</v>
+      </c>
+      <c r="G189" t="n">
+        <v>1024</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="B190" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C190" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D190" s="2" t="inlineStr">
+        <is>
+          <t>Suzuki</t>
+        </is>
+      </c>
+      <c r="E190" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F190" s="2" t="n">
+        <v>2785</v>
+      </c>
+      <c r="G190" s="2" t="n">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="B191" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C191" t="n">
+        <v>7</v>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Toyota</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F191" t="n">
+        <v>11822</v>
+      </c>
+      <c r="G191" t="n">
+        <v>1544</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8684,7 +8974,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G426"/>
+  <dimension ref="A1:G451"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -20988,6 +21278,731 @@
       </c>
       <c r="G426" s="2" t="n">
         <v>468</v>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B427" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C427" t="n">
+        <v>7</v>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>Changan</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F427" t="n">
+        <v>8510</v>
+      </c>
+      <c r="G427" t="n">
+        <v>1080</v>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B428" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C428" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D428" s="2" t="inlineStr">
+        <is>
+          <t>Chery</t>
+        </is>
+      </c>
+      <c r="E428" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F428" s="2" t="n">
+        <v>5061</v>
+      </c>
+      <c r="G428" s="2" t="n">
+        <v>797</v>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B429" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C429" t="n">
+        <v>7</v>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>Chevrolet</t>
+        </is>
+      </c>
+      <c r="E429" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F429" t="n">
+        <v>9434</v>
+      </c>
+      <c r="G429" t="n">
+        <v>1208</v>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B430" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C430" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D430" s="2" t="inlineStr">
+        <is>
+          <t>Citroen</t>
+        </is>
+      </c>
+      <c r="E430" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F430" s="2" t="n">
+        <v>2498</v>
+      </c>
+      <c r="G430" s="2" t="n">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B431" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C431" t="n">
+        <v>7</v>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>Ford</t>
+        </is>
+      </c>
+      <c r="E431" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F431" t="n">
+        <v>8961</v>
+      </c>
+      <c r="G431" t="n">
+        <v>1119</v>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B432" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C432" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D432" s="2" t="inlineStr">
+        <is>
+          <t>Foton</t>
+        </is>
+      </c>
+      <c r="E432" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F432" s="2" t="n">
+        <v>3842</v>
+      </c>
+      <c r="G432" s="2" t="n">
+        <v>644</v>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B433" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C433" t="n">
+        <v>7</v>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>Geely</t>
+        </is>
+      </c>
+      <c r="E433" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F433" t="n">
+        <v>3492</v>
+      </c>
+      <c r="G433" t="n">
+        <v>514</v>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B434" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C434" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D434" s="2" t="inlineStr">
+        <is>
+          <t>Great Wall</t>
+        </is>
+      </c>
+      <c r="E434" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F434" s="2" t="n">
+        <v>9325</v>
+      </c>
+      <c r="G434" s="2" t="n">
+        <v>1291</v>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B435" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C435" t="n">
+        <v>7</v>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>Hyundai</t>
+        </is>
+      </c>
+      <c r="E435" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F435" t="n">
+        <v>11894</v>
+      </c>
+      <c r="G435" t="n">
+        <v>1832</v>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B436" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C436" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D436" s="2" t="inlineStr">
+        <is>
+          <t>Jac</t>
+        </is>
+      </c>
+      <c r="E436" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F436" s="2" t="n">
+        <v>3782</v>
+      </c>
+      <c r="G436" s="2" t="n">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B437" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C437" t="n">
+        <v>7</v>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>Jeep</t>
+        </is>
+      </c>
+      <c r="E437" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F437" t="n">
+        <v>1924</v>
+      </c>
+      <c r="G437" t="n">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B438" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C438" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D438" s="2" t="inlineStr">
+        <is>
+          <t>Jetour</t>
+        </is>
+      </c>
+      <c r="E438" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F438" s="2" t="n">
+        <v>4377</v>
+      </c>
+      <c r="G438" s="2" t="n">
+        <v>707</v>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B439" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C439" t="n">
+        <v>7</v>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>Kia</t>
+        </is>
+      </c>
+      <c r="E439" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F439" t="n">
+        <v>10845</v>
+      </c>
+      <c r="G439" t="n">
+        <v>1850</v>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B440" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C440" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D440" s="2" t="inlineStr">
+        <is>
+          <t>Maxus</t>
+        </is>
+      </c>
+      <c r="E440" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F440" s="2" t="n">
+        <v>3522</v>
+      </c>
+      <c r="G440" s="2" t="n">
+        <v>520</v>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B441" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C441" t="n">
+        <v>7</v>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>Mazda</t>
+        </is>
+      </c>
+      <c r="E441" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F441" t="n">
+        <v>5329</v>
+      </c>
+      <c r="G441" t="n">
+        <v>737</v>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B442" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C442" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D442" s="2" t="inlineStr">
+        <is>
+          <t>Mg</t>
+        </is>
+      </c>
+      <c r="E442" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F442" s="2" t="n">
+        <v>6693</v>
+      </c>
+      <c r="G442" s="2" t="n">
+        <v>985</v>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B443" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C443" t="n">
+        <v>7</v>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>Mitsubishi</t>
+        </is>
+      </c>
+      <c r="E443" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F443" t="n">
+        <v>6725</v>
+      </c>
+      <c r="G443" t="n">
+        <v>814</v>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B444" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C444" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D444" s="2" t="inlineStr">
+        <is>
+          <t>Omoda</t>
+        </is>
+      </c>
+      <c r="E444" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F444" s="2" t="n">
+        <v>2975</v>
+      </c>
+      <c r="G444" s="2" t="n">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B445" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C445" t="n">
+        <v>7</v>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>Peugeot</t>
+        </is>
+      </c>
+      <c r="E445" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F445" t="n">
+        <v>7619</v>
+      </c>
+      <c r="G445" t="n">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B446" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C446" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D446" s="2" t="inlineStr">
+        <is>
+          <t>Ram</t>
+        </is>
+      </c>
+      <c r="E446" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F446" s="2" t="n">
+        <v>2590</v>
+      </c>
+      <c r="G446" s="2" t="n">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B447" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C447" t="n">
+        <v>7</v>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>Subaru</t>
+        </is>
+      </c>
+      <c r="E447" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F447" t="n">
+        <v>3700</v>
+      </c>
+      <c r="G447" t="n">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B448" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C448" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D448" s="2" t="inlineStr">
+        <is>
+          <t>Suzuki</t>
+        </is>
+      </c>
+      <c r="E448" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F448" s="2" t="n">
+        <v>13255</v>
+      </c>
+      <c r="G448" s="2" t="n">
+        <v>1473</v>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B449" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C449" t="n">
+        <v>7</v>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>Tesla</t>
+        </is>
+      </c>
+      <c r="E449" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F449" t="n">
+        <v>1946</v>
+      </c>
+      <c r="G449" t="n">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B450" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C450" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D450" s="2" t="inlineStr">
+        <is>
+          <t>Toyota</t>
+        </is>
+      </c>
+      <c r="E450" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F450" s="2" t="n">
+        <v>14744</v>
+      </c>
+      <c r="G450" s="2" t="n">
+        <v>2087</v>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B451" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C451" t="n">
+        <v>7</v>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="E451" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F451" t="n">
+        <v>4229</v>
+      </c>
+      <c r="G451" t="n">
+        <v>592</v>
       </c>
     </row>
   </sheetData>
@@ -38250,7 +39265,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G333"/>
+  <dimension ref="A1:G351"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -47925,6 +48940,528 @@
       </c>
       <c r="G333" t="n">
         <v>1079</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="2" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B334" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C334" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D334" s="2" t="inlineStr">
+        <is>
+          <t>Bmw</t>
+        </is>
+      </c>
+      <c r="E334" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F334" s="2" t="n">
+        <v>1183</v>
+      </c>
+      <c r="G334" s="2" t="n">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B335" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C335" t="n">
+        <v>7</v>
+      </c>
+      <c r="D335" t="inlineStr">
+        <is>
+          <t>Byd</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F335" t="n">
+        <v>7101</v>
+      </c>
+      <c r="G335" t="n">
+        <v>983</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="2" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B336" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C336" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D336" s="2" t="inlineStr">
+        <is>
+          <t>Chery</t>
+        </is>
+      </c>
+      <c r="E336" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F336" s="2" t="n">
+        <v>2840</v>
+      </c>
+      <c r="G336" s="2" t="n">
+        <v>428</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B337" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C337" t="n">
+        <v>7</v>
+      </c>
+      <c r="D337" t="inlineStr">
+        <is>
+          <t>Chevrolet</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F337" t="n">
+        <v>13998</v>
+      </c>
+      <c r="G337" t="n">
+        <v>1875</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="2" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B338" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C338" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D338" s="2" t="inlineStr">
+        <is>
+          <t>Citroen</t>
+        </is>
+      </c>
+      <c r="E338" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F338" s="2" t="n">
+        <v>1631</v>
+      </c>
+      <c r="G338" s="2" t="n">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B339" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C339" t="n">
+        <v>7</v>
+      </c>
+      <c r="D339" t="inlineStr">
+        <is>
+          <t>Dongfeng</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F339" t="n">
+        <v>2053</v>
+      </c>
+      <c r="G339" t="n">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="2" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B340" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C340" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D340" s="2" t="inlineStr">
+        <is>
+          <t>Ford</t>
+        </is>
+      </c>
+      <c r="E340" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F340" s="2" t="n">
+        <v>4987</v>
+      </c>
+      <c r="G340" s="2" t="n">
+        <v>632</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B341" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C341" t="n">
+        <v>7</v>
+      </c>
+      <c r="D341" t="inlineStr">
+        <is>
+          <t>Foton</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F341" t="n">
+        <v>4888</v>
+      </c>
+      <c r="G341" t="n">
+        <v>509</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="2" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B342" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C342" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D342" s="2" t="inlineStr">
+        <is>
+          <t>Hyundai</t>
+        </is>
+      </c>
+      <c r="E342" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F342" s="2" t="n">
+        <v>7958</v>
+      </c>
+      <c r="G342" s="2" t="n">
+        <v>1452</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B343" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C343" t="n">
+        <v>7</v>
+      </c>
+      <c r="D343" t="inlineStr">
+        <is>
+          <t>Kia</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F343" t="n">
+        <v>24483</v>
+      </c>
+      <c r="G343" t="n">
+        <v>4046</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="2" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B344" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C344" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D344" s="2" t="inlineStr">
+        <is>
+          <t>Mazda</t>
+        </is>
+      </c>
+      <c r="E344" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F344" s="2" t="n">
+        <v>13572</v>
+      </c>
+      <c r="G344" s="2" t="n">
+        <v>1854</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B345" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C345" t="n">
+        <v>7</v>
+      </c>
+      <c r="D345" t="inlineStr">
+        <is>
+          <t>Mercedes Benz</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F345" t="n">
+        <v>1931</v>
+      </c>
+      <c r="G345" t="n">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="2" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B346" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C346" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D346" s="2" t="inlineStr">
+        <is>
+          <t>Mg</t>
+        </is>
+      </c>
+      <c r="E346" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F346" s="2" t="n">
+        <v>1428</v>
+      </c>
+      <c r="G346" s="2" t="n">
+        <v>407</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B347" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C347" t="n">
+        <v>7</v>
+      </c>
+      <c r="D347" t="inlineStr">
+        <is>
+          <t>Nissan</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F347" t="n">
+        <v>7941</v>
+      </c>
+      <c r="G347" t="n">
+        <v>1320</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" s="2" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B348" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C348" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D348" s="2" t="inlineStr">
+        <is>
+          <t>Renault</t>
+        </is>
+      </c>
+      <c r="E348" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F348" s="2" t="n">
+        <v>18583</v>
+      </c>
+      <c r="G348" s="2" t="n">
+        <v>2747</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B349" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C349" t="n">
+        <v>7</v>
+      </c>
+      <c r="D349" t="inlineStr">
+        <is>
+          <t>Suzuki</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F349" t="n">
+        <v>10319</v>
+      </c>
+      <c r="G349" t="n">
+        <v>1882</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" s="2" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B350" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C350" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D350" s="2" t="inlineStr">
+        <is>
+          <t>Toyota</t>
+        </is>
+      </c>
+      <c r="E350" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F350" s="2" t="n">
+        <v>15916</v>
+      </c>
+      <c r="G350" s="2" t="n">
+        <v>3200</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B351" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C351" t="n">
+        <v>7</v>
+      </c>
+      <c r="D351" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F351" t="n">
+        <v>7374</v>
+      </c>
+      <c r="G351" t="n">
+        <v>1125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore: actualización automática 2026-09-01
</commit_message>
<xml_diff>
--- a/Base_Andina_Ventas_Auto.xlsx
+++ b/Base_Andina_Ventas_Auto.xlsx
@@ -22016,7 +22016,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G604"/>
+  <dimension ref="A1:G624"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -39252,6 +39252,584 @@
       </c>
       <c r="G604" s="2" t="n">
         <v>294</v>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B605" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C605" t="n">
+        <v>7</v>
+      </c>
+      <c r="D605" t="inlineStr">
+        <is>
+          <t>Byd</t>
+        </is>
+      </c>
+      <c r="E605" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F605" t="n">
+        <v>2738</v>
+      </c>
+      <c r="G605" t="n">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B606" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C606" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D606" s="2" t="inlineStr">
+        <is>
+          <t>Changan</t>
+        </is>
+      </c>
+      <c r="E606" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F606" s="2" t="n">
+        <v>1729</v>
+      </c>
+      <c r="G606" s="2" t="n">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B607" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C607" t="n">
+        <v>7</v>
+      </c>
+      <c r="D607" t="inlineStr">
+        <is>
+          <t>Chery</t>
+        </is>
+      </c>
+      <c r="E607" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F607" t="n">
+        <v>4428</v>
+      </c>
+      <c r="G607" t="n">
+        <v>643</v>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B608" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C608" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D608" s="2" t="inlineStr">
+        <is>
+          <t>Chevrolet</t>
+        </is>
+      </c>
+      <c r="E608" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F608" s="2" t="n">
+        <v>10945</v>
+      </c>
+      <c r="G608" s="2" t="n">
+        <v>1604</v>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B609" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C609" t="n">
+        <v>7</v>
+      </c>
+      <c r="D609" t="inlineStr">
+        <is>
+          <t>Dfsk</t>
+        </is>
+      </c>
+      <c r="E609" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F609" t="n">
+        <v>2654</v>
+      </c>
+      <c r="G609" t="n">
+        <v>426</v>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B610" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C610" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D610" s="2" t="inlineStr">
+        <is>
+          <t>Dongfeng</t>
+        </is>
+      </c>
+      <c r="E610" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F610" s="2" t="n">
+        <v>3553</v>
+      </c>
+      <c r="G610" s="2" t="n">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B611" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C611" t="n">
+        <v>7</v>
+      </c>
+      <c r="D611" t="inlineStr">
+        <is>
+          <t>Ford</t>
+        </is>
+      </c>
+      <c r="E611" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F611" t="n">
+        <v>1220</v>
+      </c>
+      <c r="G611" t="inlineStr"/>
+    </row>
+    <row r="612">
+      <c r="A612" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B612" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C612" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D612" s="2" t="inlineStr">
+        <is>
+          <t>Foton</t>
+        </is>
+      </c>
+      <c r="E612" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F612" s="2" t="n">
+        <v>1638</v>
+      </c>
+      <c r="G612" s="2" t="n">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B613" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C613" t="n">
+        <v>7</v>
+      </c>
+      <c r="D613" t="inlineStr">
+        <is>
+          <t>Great Wall</t>
+        </is>
+      </c>
+      <c r="E613" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F613" t="n">
+        <v>5095</v>
+      </c>
+      <c r="G613" t="n">
+        <v>766</v>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B614" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C614" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D614" s="2" t="inlineStr">
+        <is>
+          <t>Hino</t>
+        </is>
+      </c>
+      <c r="E614" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F614" s="2" t="n">
+        <v>1235</v>
+      </c>
+      <c r="G614" s="2" t="n">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B615" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C615" t="n">
+        <v>7</v>
+      </c>
+      <c r="D615" t="inlineStr">
+        <is>
+          <t>Hyundai</t>
+        </is>
+      </c>
+      <c r="E615" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F615" t="n">
+        <v>4969</v>
+      </c>
+      <c r="G615" t="n">
+        <v>737</v>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B616" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C616" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D616" s="2" t="inlineStr">
+        <is>
+          <t>Jac</t>
+        </is>
+      </c>
+      <c r="E616" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F616" s="2" t="n">
+        <v>3270</v>
+      </c>
+      <c r="G616" s="2" t="n">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B617" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C617" t="n">
+        <v>7</v>
+      </c>
+      <c r="D617" t="inlineStr">
+        <is>
+          <t>Jetour</t>
+        </is>
+      </c>
+      <c r="E617" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F617" t="n">
+        <v>2119</v>
+      </c>
+      <c r="G617" t="n">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B618" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C618" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D618" s="2" t="inlineStr">
+        <is>
+          <t>Kia</t>
+        </is>
+      </c>
+      <c r="E618" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F618" s="2" t="n">
+        <v>14855</v>
+      </c>
+      <c r="G618" s="2" t="n">
+        <v>2343</v>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B619" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C619" t="n">
+        <v>7</v>
+      </c>
+      <c r="D619" t="inlineStr">
+        <is>
+          <t>Mazda</t>
+        </is>
+      </c>
+      <c r="E619" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F619" t="n">
+        <v>2017</v>
+      </c>
+      <c r="G619" t="n">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B620" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C620" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D620" s="2" t="inlineStr">
+        <is>
+          <t>Mg</t>
+        </is>
+      </c>
+      <c r="E620" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F620" s="2" t="n">
+        <v>1259</v>
+      </c>
+      <c r="G620" s="2" t="n">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B621" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C621" t="n">
+        <v>7</v>
+      </c>
+      <c r="D621" t="inlineStr">
+        <is>
+          <t>Sinotruk</t>
+        </is>
+      </c>
+      <c r="E621" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F621" t="n">
+        <v>2977</v>
+      </c>
+      <c r="G621" t="n">
+        <v>406</v>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B622" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C622" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D622" s="2" t="inlineStr">
+        <is>
+          <t>Suzuki</t>
+        </is>
+      </c>
+      <c r="E622" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F622" s="2" t="n">
+        <v>2918</v>
+      </c>
+      <c r="G622" s="2" t="n">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B623" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C623" t="n">
+        <v>7</v>
+      </c>
+      <c r="D623" t="inlineStr">
+        <is>
+          <t>Toyota</t>
+        </is>
+      </c>
+      <c r="E623" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F623" t="n">
+        <v>4662</v>
+      </c>
+      <c r="G623" t="n">
+        <v>854</v>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" s="2" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="B624" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C624" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D624" s="2" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="E624" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F624" s="2" t="n">
+        <v>1926</v>
+      </c>
+      <c r="G624" s="2" t="n">
+        <v>310</v>
       </c>
     </row>
   </sheetData>
@@ -49475,7 +50053,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G70"/>
+  <dimension ref="A1:G90"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -51210,14 +51788,14 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Rep. Dominicana</t>
+          <t>Guatemala</t>
         </is>
       </c>
       <c r="B61" t="n">
         <v>2026</v>
       </c>
       <c r="C61" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D61" t="inlineStr">
         <is>
@@ -51230,52 +51808,56 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>1155</v>
-      </c>
-      <c r="G61" t="inlineStr"/>
+        <v>2136</v>
+      </c>
+      <c r="G61" t="n">
+        <v>294</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>Rep. Dominicana</t>
+          <t>Guatemala</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
         <v>2026</v>
       </c>
       <c r="C62" s="2" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>Chevrolet</t>
+          <t>Foton</t>
         </is>
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F62" s="2" t="n">
-        <v>728</v>
-      </c>
-      <c r="G62" s="2" t="inlineStr"/>
+        <v>1629</v>
+      </c>
+      <c r="G62" s="2" t="n">
+        <v>182</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Rep. Dominicana</t>
+          <t>Guatemala</t>
         </is>
       </c>
       <c r="B63" t="n">
         <v>2026</v>
       </c>
       <c r="C63" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Honda</t>
+          <t>Hino</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -51284,25 +51866,27 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>475</v>
-      </c>
-      <c r="G63" t="inlineStr"/>
+        <v>1754</v>
+      </c>
+      <c r="G63" t="n">
+        <v>253</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Rep. Dominicana</t>
+          <t>Guatemala</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
         <v>2026</v>
       </c>
       <c r="C64" s="2" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>Hyundai</t>
+          <t>Isuzu</t>
         </is>
       </c>
       <c r="E64" s="2" t="inlineStr">
@@ -51311,79 +51895,85 @@
         </is>
       </c>
       <c r="F64" s="2" t="n">
-        <v>1618</v>
-      </c>
-      <c r="G64" s="2" t="inlineStr"/>
+        <v>4380</v>
+      </c>
+      <c r="G64" s="2" t="n">
+        <v>707</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Rep. Dominicana</t>
+          <t>Guatemala</t>
         </is>
       </c>
       <c r="B65" t="n">
         <v>2026</v>
       </c>
       <c r="C65" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Isuzu</t>
+          <t>Jac</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Otra</t>
+          <t>China 🇨🇳</t>
         </is>
       </c>
       <c r="F65" t="n">
-        <v>1292</v>
-      </c>
-      <c r="G65" t="inlineStr"/>
+        <v>2638</v>
+      </c>
+      <c r="G65" t="n">
+        <v>434</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Rep. Dominicana</t>
+          <t>Guatemala</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
         <v>2026</v>
       </c>
       <c r="C66" s="2" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Jetour</t>
+          <t>Kia</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>China 🇨🇳</t>
+          <t>Otra</t>
         </is>
       </c>
       <c r="F66" s="2" t="n">
-        <v>469</v>
-      </c>
-      <c r="G66" s="2" t="inlineStr"/>
+        <v>2156</v>
+      </c>
+      <c r="G66" s="2" t="n">
+        <v>293</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Rep. Dominicana</t>
+          <t>Guatemala</t>
         </is>
       </c>
       <c r="B67" t="n">
         <v>2026</v>
       </c>
       <c r="C67" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Kia</t>
+          <t>Mitsubishi</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -51392,25 +51982,27 @@
         </is>
       </c>
       <c r="F67" t="n">
-        <v>1566</v>
-      </c>
-      <c r="G67" t="inlineStr"/>
+        <v>2752</v>
+      </c>
+      <c r="G67" t="n">
+        <v>469</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>Rep. Dominicana</t>
+          <t>Guatemala</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
         <v>2026</v>
       </c>
       <c r="C68" s="2" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>Nissan</t>
+          <t>Suzuki</t>
         </is>
       </c>
       <c r="E68" s="2" t="inlineStr">
@@ -51419,25 +52011,27 @@
         </is>
       </c>
       <c r="F68" s="2" t="n">
-        <v>657</v>
-      </c>
-      <c r="G68" s="2" t="inlineStr"/>
+        <v>2409</v>
+      </c>
+      <c r="G68" s="2" t="n">
+        <v>430</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Rep. Dominicana</t>
+          <t>Guatemala</t>
         </is>
       </c>
       <c r="B69" t="n">
         <v>2026</v>
       </c>
       <c r="C69" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Suzuki</t>
+          <t>Toyota</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -51446,36 +52040,580 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>831</v>
-      </c>
-      <c r="G69" t="inlineStr"/>
+        <v>10776</v>
+      </c>
+      <c r="G69" t="n">
+        <v>1613</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
+          <t>Guatemala</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C70" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="n">
+        <v>1196</v>
+      </c>
+      <c r="G70" s="2" t="n">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
           <t>Rep. Dominicana</t>
         </is>
       </c>
-      <c r="B70" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="C70" s="2" t="n">
+      <c r="B71" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C71" t="n">
         <v>5</v>
       </c>
-      <c r="D70" s="2" t="inlineStr">
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Changan</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F71" t="n">
+        <v>1155</v>
+      </c>
+      <c r="G71" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>Rep. Dominicana</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C72" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>Chevrolet</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="n">
+        <v>728</v>
+      </c>
+      <c r="G72" s="2" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Rep. Dominicana</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C73" t="n">
+        <v>5</v>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Honda</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F73" t="n">
+        <v>475</v>
+      </c>
+      <c r="G73" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>Rep. Dominicana</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C74" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>Hyundai</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="n">
+        <v>1618</v>
+      </c>
+      <c r="G74" s="2" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Rep. Dominicana</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C75" t="n">
+        <v>5</v>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Isuzu</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>1292</v>
+      </c>
+      <c r="G75" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>Rep. Dominicana</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C76" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>Jetour</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="n">
+        <v>469</v>
+      </c>
+      <c r="G76" s="2" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Rep. Dominicana</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C77" t="n">
+        <v>5</v>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>Kia</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>1566</v>
+      </c>
+      <c r="G77" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>Rep. Dominicana</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C78" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>Nissan</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="n">
+        <v>657</v>
+      </c>
+      <c r="G78" s="2" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Rep. Dominicana</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C79" t="n">
+        <v>5</v>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>Suzuki</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>831</v>
+      </c>
+      <c r="G79" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>Rep. Dominicana</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C80" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
         <is>
           <t>Toyota</t>
         </is>
       </c>
-      <c r="E70" s="2" t="inlineStr">
-        <is>
-          <t>Otra</t>
-        </is>
-      </c>
-      <c r="F70" s="2" t="n">
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="n">
         <v>2304</v>
       </c>
-      <c r="G70" s="2" t="inlineStr"/>
+      <c r="G80" s="2" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Rep. Dominicana</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C81" t="n">
+        <v>7</v>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Changan</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F81" t="n">
+        <v>1671</v>
+      </c>
+      <c r="G81" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Rep. Dominicana</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C82" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>Chevrolet</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="n">
+        <v>1093</v>
+      </c>
+      <c r="G82" s="2" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Rep. Dominicana</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C83" t="n">
+        <v>7</v>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Geely</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F83" t="n">
+        <v>801</v>
+      </c>
+      <c r="G83" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>Rep. Dominicana</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C84" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>Hyundai</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="n">
+        <v>2210</v>
+      </c>
+      <c r="G84" s="2" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Rep. Dominicana</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C85" t="n">
+        <v>7</v>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>Isuzu</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F85" t="n">
+        <v>1944</v>
+      </c>
+      <c r="G85" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>Rep. Dominicana</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C86" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>Jetour</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="n">
+        <v>767</v>
+      </c>
+      <c r="G86" s="2" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Rep. Dominicana</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C87" t="n">
+        <v>7</v>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Kia</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F87" t="n">
+        <v>2840</v>
+      </c>
+      <c r="G87" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>Rep. Dominicana</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C88" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>Nissan</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="n">
+        <v>1095</v>
+      </c>
+      <c r="G88" s="2" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Rep. Dominicana</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C89" t="n">
+        <v>7</v>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Suzuki</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F89" t="n">
+        <v>1288</v>
+      </c>
+      <c r="G89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>Rep. Dominicana</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C90" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>Toyota</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="n">
+        <v>3481</v>
+      </c>
+      <c r="G90" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore: actualización automática 2026-09-15
</commit_message>
<xml_diff>
--- a/Base_Andina_Ventas_Auto.xlsx
+++ b/Base_Andina_Ventas_Auto.xlsx
@@ -3414,7 +3414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G191"/>
+  <dimension ref="A1:G201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -8963,6 +8963,296 @@
         <v>1544</v>
       </c>
     </row>
+    <row r="192">
+      <c r="A192" s="2" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="B192" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C192" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D192" s="2" t="inlineStr">
+        <is>
+          <t>Changan</t>
+        </is>
+      </c>
+      <c r="E192" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F192" s="2" t="n">
+        <v>5750</v>
+      </c>
+      <c r="G192" s="2" t="n">
+        <v>818</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="B193" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C193" t="n">
+        <v>8</v>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Chery</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F193" t="n">
+        <v>4457</v>
+      </c>
+      <c r="G193" t="n">
+        <v>685</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="B194" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C194" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D194" s="2" t="inlineStr">
+        <is>
+          <t>Ford</t>
+        </is>
+      </c>
+      <c r="E194" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F194" s="2" t="n">
+        <v>4261</v>
+      </c>
+      <c r="G194" s="2" t="n">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="B195" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C195" t="n">
+        <v>8</v>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>Geely</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F195" t="n">
+        <v>7131</v>
+      </c>
+      <c r="G195" t="n">
+        <v>1074</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="B196" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C196" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D196" s="2" t="inlineStr">
+        <is>
+          <t>Hyundai</t>
+        </is>
+      </c>
+      <c r="E196" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F196" s="2" t="n">
+        <v>7562</v>
+      </c>
+      <c r="G196" s="2" t="n">
+        <v>992</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="B197" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C197" t="n">
+        <v>8</v>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Jac</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F197" t="n">
+        <v>3020</v>
+      </c>
+      <c r="G197" t="n">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="B198" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C198" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D198" s="2" t="inlineStr">
+        <is>
+          <t>Jetour</t>
+        </is>
+      </c>
+      <c r="E198" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F198" s="2" t="n">
+        <v>10326</v>
+      </c>
+      <c r="G198" s="2" t="n">
+        <v>1685</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="B199" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C199" t="n">
+        <v>8</v>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Kia</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F199" t="n">
+        <v>7921</v>
+      </c>
+      <c r="G199" t="n">
+        <v>1304</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="B200" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C200" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D200" s="2" t="inlineStr">
+        <is>
+          <t>Suzuki</t>
+        </is>
+      </c>
+      <c r="E200" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F200" s="2" t="n">
+        <v>3275</v>
+      </c>
+      <c r="G200" s="2" t="n">
+        <v>490</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>Peru</t>
+        </is>
+      </c>
+      <c r="B201" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C201" t="n">
+        <v>8</v>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Toyota</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F201" t="n">
+        <v>13826</v>
+      </c>
+      <c r="G201" t="n">
+        <v>2004</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -8974,7 +9264,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G451"/>
+  <dimension ref="A1:G476"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -22003,6 +22293,731 @@
       </c>
       <c r="G451" t="n">
         <v>592</v>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B452" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C452" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D452" s="2" t="inlineStr">
+        <is>
+          <t>Changan</t>
+        </is>
+      </c>
+      <c r="E452" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F452" s="2" t="n">
+        <v>9547</v>
+      </c>
+      <c r="G452" s="2" t="n">
+        <v>1037</v>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B453" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C453" t="n">
+        <v>8</v>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>Chery</t>
+        </is>
+      </c>
+      <c r="E453" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F453" t="n">
+        <v>5966</v>
+      </c>
+      <c r="G453" t="n">
+        <v>905</v>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B454" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C454" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D454" s="2" t="inlineStr">
+        <is>
+          <t>Chevrolet</t>
+        </is>
+      </c>
+      <c r="E454" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F454" s="2" t="n">
+        <v>11012</v>
+      </c>
+      <c r="G454" s="2" t="n">
+        <v>1578</v>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B455" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C455" t="n">
+        <v>8</v>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>Citroen</t>
+        </is>
+      </c>
+      <c r="E455" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F455" t="n">
+        <v>2824</v>
+      </c>
+      <c r="G455" t="n">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B456" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C456" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D456" s="2" t="inlineStr">
+        <is>
+          <t>Ford</t>
+        </is>
+      </c>
+      <c r="E456" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F456" s="2" t="n">
+        <v>10300</v>
+      </c>
+      <c r="G456" s="2" t="n">
+        <v>1339</v>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B457" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C457" t="n">
+        <v>8</v>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>Foton</t>
+        </is>
+      </c>
+      <c r="E457" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F457" t="n">
+        <v>4597</v>
+      </c>
+      <c r="G457" t="n">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B458" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C458" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D458" s="2" t="inlineStr">
+        <is>
+          <t>Geely</t>
+        </is>
+      </c>
+      <c r="E458" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F458" s="2" t="n">
+        <v>4046</v>
+      </c>
+      <c r="G458" s="2" t="n">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B459" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C459" t="n">
+        <v>8</v>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>Great Wall</t>
+        </is>
+      </c>
+      <c r="E459" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F459" t="n">
+        <v>10430</v>
+      </c>
+      <c r="G459" t="n">
+        <v>1105</v>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B460" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C460" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D460" s="2" t="inlineStr">
+        <is>
+          <t>Hyundai</t>
+        </is>
+      </c>
+      <c r="E460" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F460" s="2" t="n">
+        <v>14246</v>
+      </c>
+      <c r="G460" s="2" t="n">
+        <v>2352</v>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B461" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C461" t="n">
+        <v>8</v>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>Jac</t>
+        </is>
+      </c>
+      <c r="E461" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F461" t="n">
+        <v>4376</v>
+      </c>
+      <c r="G461" t="n">
+        <v>594</v>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B462" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C462" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D462" s="2" t="inlineStr">
+        <is>
+          <t>Jeep</t>
+        </is>
+      </c>
+      <c r="E462" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F462" s="2" t="n">
+        <v>2212</v>
+      </c>
+      <c r="G462" s="2" t="n">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B463" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C463" t="n">
+        <v>8</v>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>Jetour</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F463" t="n">
+        <v>5175</v>
+      </c>
+      <c r="G463" t="n">
+        <v>798</v>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B464" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C464" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D464" s="2" t="inlineStr">
+        <is>
+          <t>Kia</t>
+        </is>
+      </c>
+      <c r="E464" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F464" s="2" t="n">
+        <v>12918</v>
+      </c>
+      <c r="G464" s="2" t="n">
+        <v>2073</v>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B465" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C465" t="n">
+        <v>8</v>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>Maxus</t>
+        </is>
+      </c>
+      <c r="E465" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F465" t="n">
+        <v>3916</v>
+      </c>
+      <c r="G465" t="n">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B466" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C466" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D466" s="2" t="inlineStr">
+        <is>
+          <t>Mazda</t>
+        </is>
+      </c>
+      <c r="E466" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F466" s="2" t="n">
+        <v>6296</v>
+      </c>
+      <c r="G466" s="2" t="n">
+        <v>967</v>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B467" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C467" t="n">
+        <v>8</v>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>Mg</t>
+        </is>
+      </c>
+      <c r="E467" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F467" t="n">
+        <v>7452</v>
+      </c>
+      <c r="G467" t="n">
+        <v>759</v>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B468" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C468" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D468" s="2" t="inlineStr">
+        <is>
+          <t>Mitsubishi</t>
+        </is>
+      </c>
+      <c r="E468" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F468" s="2" t="n">
+        <v>7349</v>
+      </c>
+      <c r="G468" s="2" t="n">
+        <v>624</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B469" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C469" t="n">
+        <v>8</v>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>Omoda</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F469" t="n">
+        <v>3426</v>
+      </c>
+      <c r="G469" t="n">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B470" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C470" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D470" s="2" t="inlineStr">
+        <is>
+          <t>Peugeot</t>
+        </is>
+      </c>
+      <c r="E470" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F470" s="2" t="n">
+        <v>8625</v>
+      </c>
+      <c r="G470" s="2" t="n">
+        <v>1006</v>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B471" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C471" t="n">
+        <v>8</v>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>Ram</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F471" t="n">
+        <v>3036</v>
+      </c>
+      <c r="G471" t="n">
+        <v>446</v>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B472" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C472" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D472" s="2" t="inlineStr">
+        <is>
+          <t>Subaru</t>
+        </is>
+      </c>
+      <c r="E472" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F472" s="2" t="n">
+        <v>4445</v>
+      </c>
+      <c r="G472" s="2" t="n">
+        <v>745</v>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B473" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C473" t="n">
+        <v>8</v>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>Suzuki</t>
+        </is>
+      </c>
+      <c r="E473" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F473" t="n">
+        <v>15006</v>
+      </c>
+      <c r="G473" t="n">
+        <v>1751</v>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B474" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C474" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D474" s="2" t="inlineStr">
+        <is>
+          <t>Tesla</t>
+        </is>
+      </c>
+      <c r="E474" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F474" s="2" t="n">
+        <v>2412</v>
+      </c>
+      <c r="G474" s="2" t="n">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B475" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C475" t="n">
+        <v>8</v>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>Toyota</t>
+        </is>
+      </c>
+      <c r="E475" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F475" t="n">
+        <v>17858</v>
+      </c>
+      <c r="G475" t="n">
+        <v>3114</v>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="B476" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C476" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D476" s="2" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="E476" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F476" s="2" t="n">
+        <v>4879</v>
+      </c>
+      <c r="G476" s="2" t="n">
+        <v>650</v>
       </c>
     </row>
   </sheetData>
@@ -39843,7 +40858,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G351"/>
+  <dimension ref="A1:G369"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -50040,6 +51055,528 @@
       </c>
       <c r="G351" t="n">
         <v>1125</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="2" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B352" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C352" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D352" s="2" t="inlineStr">
+        <is>
+          <t>Bmw</t>
+        </is>
+      </c>
+      <c r="E352" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F352" s="2" t="n">
+        <v>1438</v>
+      </c>
+      <c r="G352" s="2" t="n">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B353" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C353" t="n">
+        <v>8</v>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>Byd</t>
+        </is>
+      </c>
+      <c r="E353" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F353" t="n">
+        <v>8127</v>
+      </c>
+      <c r="G353" t="n">
+        <v>1026</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="2" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B354" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C354" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D354" s="2" t="inlineStr">
+        <is>
+          <t>Chery</t>
+        </is>
+      </c>
+      <c r="E354" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F354" s="2" t="n">
+        <v>3198</v>
+      </c>
+      <c r="G354" s="2" t="n">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B355" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C355" t="n">
+        <v>8</v>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>Chevrolet</t>
+        </is>
+      </c>
+      <c r="E355" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F355" t="n">
+        <v>15782</v>
+      </c>
+      <c r="G355" t="n">
+        <v>1784</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" s="2" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B356" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C356" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D356" s="2" t="inlineStr">
+        <is>
+          <t>Citroen</t>
+        </is>
+      </c>
+      <c r="E356" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F356" s="2" t="n">
+        <v>1852</v>
+      </c>
+      <c r="G356" s="2" t="n">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B357" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C357" t="n">
+        <v>8</v>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>Deepal</t>
+        </is>
+      </c>
+      <c r="E357" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F357" t="n">
+        <v>245</v>
+      </c>
+      <c r="G357" t="n">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="2" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B358" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C358" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D358" s="2" t="inlineStr">
+        <is>
+          <t>Ford</t>
+        </is>
+      </c>
+      <c r="E358" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F358" s="2" t="n">
+        <v>6019</v>
+      </c>
+      <c r="G358" s="2" t="n">
+        <v>1032</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B359" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C359" t="n">
+        <v>8</v>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>Foton</t>
+        </is>
+      </c>
+      <c r="E359" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F359" t="n">
+        <v>5288</v>
+      </c>
+      <c r="G359" t="n">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="2" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B360" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C360" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D360" s="2" t="inlineStr">
+        <is>
+          <t>Hyundai</t>
+        </is>
+      </c>
+      <c r="E360" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F360" s="2" t="n">
+        <v>9139</v>
+      </c>
+      <c r="G360" s="2" t="n">
+        <v>1181</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B361" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C361" t="n">
+        <v>8</v>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>Kia</t>
+        </is>
+      </c>
+      <c r="E361" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F361" t="n">
+        <v>28077</v>
+      </c>
+      <c r="G361" t="n">
+        <v>3594</v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" s="2" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B362" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C362" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D362" s="2" t="inlineStr">
+        <is>
+          <t>Mazda</t>
+        </is>
+      </c>
+      <c r="E362" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F362" s="2" t="n">
+        <v>15281</v>
+      </c>
+      <c r="G362" s="2" t="n">
+        <v>1709</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B363" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C363" t="n">
+        <v>8</v>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>Mercedes Benz</t>
+        </is>
+      </c>
+      <c r="E363" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F363" t="n">
+        <v>2156</v>
+      </c>
+      <c r="G363" t="n">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" s="2" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B364" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C364" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D364" s="2" t="inlineStr">
+        <is>
+          <t>Mg</t>
+        </is>
+      </c>
+      <c r="E364" s="2" t="inlineStr">
+        <is>
+          <t>China 🇨🇳</t>
+        </is>
+      </c>
+      <c r="F364" s="2" t="n">
+        <v>1884</v>
+      </c>
+      <c r="G364" s="2" t="n">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B365" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C365" t="n">
+        <v>8</v>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>Nissan</t>
+        </is>
+      </c>
+      <c r="E365" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F365" t="n">
+        <v>9402</v>
+      </c>
+      <c r="G365" t="n">
+        <v>1461</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="2" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B366" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C366" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D366" s="2" t="inlineStr">
+        <is>
+          <t>Renault</t>
+        </is>
+      </c>
+      <c r="E366" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F366" s="2" t="n">
+        <v>21266</v>
+      </c>
+      <c r="G366" s="2" t="n">
+        <v>2683</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B367" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C367" t="n">
+        <v>8</v>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>Suzuki</t>
+        </is>
+      </c>
+      <c r="E367" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F367" t="n">
+        <v>11695</v>
+      </c>
+      <c r="G367" t="n">
+        <v>1376</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="2" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B368" s="2" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C368" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="D368" s="2" t="inlineStr">
+        <is>
+          <t>Toyota</t>
+        </is>
+      </c>
+      <c r="E368" s="2" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F368" s="2" t="n">
+        <v>18946</v>
+      </c>
+      <c r="G368" s="2" t="n">
+        <v>3030</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>Colombia</t>
+        </is>
+      </c>
+      <c r="B369" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C369" t="n">
+        <v>8</v>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>Volkswagen</t>
+        </is>
+      </c>
+      <c r="E369" t="inlineStr">
+        <is>
+          <t>Otra</t>
+        </is>
+      </c>
+      <c r="F369" t="n">
+        <v>8377</v>
+      </c>
+      <c r="G369" t="n">
+        <v>1003</v>
       </c>
     </row>
   </sheetData>

</xml_diff>